<commit_message>
Update berita 2026-08-03 23:57 UTC
</commit_message>
<xml_diff>
--- a/data/berita_antara_2026-07-28.xlsx
+++ b/data/berita_antara_2026-07-28.xlsx
@@ -476,259 +476,259 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paspor habis masa berlaku? Begini cara perpanjang, syarat, dan biaya terbarunya</t>
+          <t>Apakah pindah rumah wajib ganti KTP dan KK?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 07:06:24 +0700</t>
+          <t>Tue, 28 Jul 2026 05:58:39 +0700</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Paspor merupakan dokumen resmi yang diterbitkan pemerintah sebagai bukti identitas dan kewarganegaraan seseorang saat ...</t>
+          <t>Masyarakat yang pindah rumah atau tinggal di rumah kontrakan kerap bertanya apakah wajib mengubah alamat pada Kartu ...</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668629/paspor-habis-masa-berlaku-begini-cara-perpanjang-syarat-dan-biaya-terbarunya</t>
+          <t>https://www.antaranews.com/berita/5668575/apakah-pindah-rumah-wajib-ganti-ktp-dan-kk</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/Imigrasi-CFD.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/capil.jpeg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>politik</t>
+          <t>sepakbola</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Apakah pindah rumah wajib ganti KTP dan KK?</t>
+          <t>9 rekor Piala AFF yang masih bertahan hingga kini, Indonesia masuk daftar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 05:58:39 +0700</t>
+          <t>Tue, 28 Jul 2026 06:50:07 +0700</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Masyarakat yang pindah rumah atau tinggal di rumah kontrakan kerap bertanya apakah wajib mengubah alamat pada Kartu ...</t>
+          <t>Kejuaraan sepak bola antarnegara Asia Tenggara, ASEAN Hyundai Cup 2026 atau Piala AFF 2026, kembali menjadi panggung ...</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668575/apakah-pindah-rumah-wajib-ganti-ktp-dan-kk</t>
+          <t>https://www.antaranews.com/berita/5668612/9-rekor-piala-aff-yang-masih-bertahan-hingga-kini-indonesia-masuk-daftar</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/23/capil.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/timnas-indonesia-kalahkan-kamboja-2829197.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ekonomi</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Kenapa harga emas turun? Ini 5 penyebab utama dan prospeknya ke depan</t>
+          <t>Cara cek BPJS kesehatan aktif atau tidak lewat WhatsApp, mudah tanpa aplikasi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 08:36:17 +0700</t>
+          <t>Tue, 28 Jul 2026 06:23:21 +0700</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Emas dikenal sebagai salah satu instrumen investasi yang kerap dijadikan aset lindung nilai (safe haven), terutama ...</t>
+          <t>Peserta Jaminan Kesehatan Nasional (JKN) perlu memastikan status kepesertaan BPJS Kesehatan selalu aktif agar dapat ...</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668688/kenapa-harga-emas-turun-ini-5-penyebab-utama-dan-prospeknya-ke-depan</t>
+          <t>https://www.antaranews.com/berita/5668596/cara-cek-bpjs-kesehatan-aktif-atau-tidak-lewat-whatsapp-mudah-tanpa-aplikasi</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/bazar-emas-pegadaian-di-palu-2718730.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/WhatsApp-Image-2026-07-27-at-15.12.29.jpeg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ekonomi, otomotif</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Apakah motor listrik boleh dicas semalaman? Ini penjelasan dan tips agar baterai awet</t>
+          <t>Bansos anak balita PKH 2026: Syarat penerima, besaran bantuan, dan cara cek</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 07:00:21 +0700</t>
+          <t>Tue, 28 Jul 2026 06:11:30 +0700</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Kebiasaan mengecas motor listrik semalaman masih menjadi pertanyaan bagi banyak pengguna. Meski sebagian motor listrik ...</t>
+          <t>Pemerintah kembali menyalurkan bantuan sosial bagi keluarga yang memiliki anak usia dini melalui Program Keluarga ...</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://otomotif.antaranews.com/berita/5668623/apakah-motor-listrik-boleh-dicas-semalaman-ini-penjelasan-dan-tips-agar-baterai-awet</t>
+          <t>https://www.antaranews.com/berita/5668585/bansos-anak-balita-pkh-2026-syarat-penerima-besaran-bantuan-dan-cara-cek</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000137568.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/bltd-kota.jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sepakbola</t>
+          <t>humaniora</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>9 rekor Piala AFF yang masih bertahan hingga kini, Indonesia masuk daftar</t>
+          <t>Cara daftar Bansos Online lewat portal Perlinsos, syarat &amp; langkah-langkahnya</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 06:50:07 +0700</t>
+          <t>Tue, 28 Jul 2026 06:06:00 +0700</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kejuaraan sepak bola antarnegara Asia Tenggara, ASEAN Hyundai Cup 2026 atau Piala AFF 2026, kembali menjadi panggung ...</t>
+          <t>Pemerintah menghadirkan Portal Perlindungan Sosial (Perlinsos) untuk memudahkan masyarakat mengajukan bantuan sosial ...</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668612/9-rekor-piala-aff-yang-masih-bertahan-hingga-kini-indonesia-masuk-daftar</t>
+          <t>https://www.antaranews.com/berita/5668579/cara-daftar-bansos-online-lewat-portal-perlinsos-syarat-langkah-langkahnya</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/28/timnas-indonesia-kalahkan-kamboja-2829197.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/22/uji-coba-perlinsos-digital-di-makassar-2825760.jpg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>politik</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cara cek NISN online dengan nama, mudah dan cepat tanpa ke sekolah</t>
+          <t>Paspor habis masa berlaku? Begini cara perpanjang, syarat, dan biaya terbarunya</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 07:11:22 +0700</t>
+          <t>Tue, 28 Jul 2026 07:06:24 +0700</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Nomor Induk Siswa Nasional (NISN) merupakan identitas resmi yang dimiliki setiap peserta didik di Indonesia. Nomor ini ...</t>
+          <t>Paspor merupakan dokumen resmi yang diterbitkan pemerintah sebagai bukti identitas dan kewarganegaraan seseorang saat ...</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668635/cara-cek-nisn-online-dengan-nama-mudah-dan-cepat-tanpa-ke-sekolah</t>
+          <t>https://www.antaranews.com/berita/5668629/paspor-habis-masa-berlaku-begini-cara-perpanjang-syarat-dan-biaya-terbarunya</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2025/06/11/nisn-website.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/Imigrasi-CFD.jpeg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>ekonomi</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cara cek BPJS kesehatan aktif atau tidak lewat WhatsApp, mudah tanpa aplikasi</t>
+          <t>Kenapa harga emas turun? Ini 5 penyebab utama dan prospeknya ke depan</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 06:23:21 +0700</t>
+          <t>Tue, 28 Jul 2026 08:36:17 +0700</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Peserta Jaminan Kesehatan Nasional (JKN) perlu memastikan status kepesertaan BPJS Kesehatan selalu aktif agar dapat ...</t>
+          <t>Emas dikenal sebagai salah satu instrumen investasi yang kerap dijadikan aset lindung nilai (safe haven), terutama ...</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668596/cara-cek-bpjs-kesehatan-aktif-atau-tidak-lewat-whatsapp-mudah-tanpa-aplikasi</t>
+          <t>https://www.antaranews.com/berita/5668688/kenapa-harga-emas-turun-ini-5-penyebab-utama-dan-prospeknya-ke-depan</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/WhatsApp-Image-2026-07-27-at-15.12.29.jpeg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/bazar-emas-pegadaian-di-palu-2718730.jpg</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>humaniora</t>
+          <t>ekonomi, otomotif</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bansos anak balita PKH 2026: Syarat penerima, besaran bantuan, dan cara cek</t>
+          <t>Apakah motor listrik boleh dicas semalaman? Ini penjelasan dan tips agar baterai awet</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 06:11:30 +0700</t>
+          <t>Tue, 28 Jul 2026 07:00:21 +0700</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pemerintah kembali menyalurkan bantuan sosial bagi keluarga yang memiliki anak usia dini melalui Program Keluarga ...</t>
+          <t>Kebiasaan mengecas motor listrik semalaman masih menjadi pertanyaan bagi banyak pengguna. Meski sebagian motor listrik ...</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668585/bansos-anak-balita-pkh-2026-syarat-penerima-besaran-bantuan-dan-cara-cek</t>
+          <t>https://otomotif.antaranews.com/berita/5668623/apakah-motor-listrik-boleh-dicas-semalaman-ini-penjelasan-dan-tips-agar-baterai-awet</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/bltd-kota.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/18/1000137568.jpg</t>
         </is>
       </c>
     </row>
@@ -740,28 +740,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cara daftar Bansos Online lewat portal Perlinsos, syarat &amp; langkah-langkahnya</t>
+          <t>Cara cek NISN online dengan nama, mudah dan cepat tanpa ke sekolah</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tue, 28 Jul 2026 06:06:00 +0700</t>
+          <t>Tue, 28 Jul 2026 07:11:22 +0700</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Pemerintah menghadirkan Portal Perlindungan Sosial (Perlinsos) untuk memudahkan masyarakat mengajukan bantuan sosial ...</t>
+          <t>Nomor Induk Siswa Nasional (NISN) merupakan identitas resmi yang dimiliki setiap peserta didik di Indonesia. Nomor ini ...</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.antaranews.com/berita/5668579/cara-daftar-bansos-online-lewat-portal-perlinsos-syarat-langkah-langkahnya</t>
+          <t>https://www.antaranews.com/berita/5668635/cara-cek-nisn-online-dengan-nama-mudah-dan-cepat-tanpa-ke-sekolah</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://cdn.antaranews.com/cache/800x533/2026/07/22/uji-coba-perlinsos-digital-di-makassar-2825760.jpg</t>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/06/11/nisn-website.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>